<commit_message>
chore(data): sync daily pipeline outputs
Routine ingestion sync: odds/availability snapshots, esports match data,
model ledgers, and baseline config refreshes from the background daily
collection job.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/flat/model_ledgers/mlb-moneyline-elo-trend-lr.xlsx
+++ b/data/flat/model_ledgers/mlb-moneyline-elo-trend-lr.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Predictions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Predictions'!$A$1:$AJ$318</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Predictions'!$A$1:$AJ$331</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ318"/>
+  <dimension ref="A1:AJ331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -34874,8 +34874,1386 @@
       <c r="AI318" s="2" t="inlineStr"/>
       <c r="AJ318" s="2" t="inlineStr"/>
     </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>f8c9ab98bc8643df</t>
+        </is>
+      </c>
+      <c r="B319" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C319" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E319" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F319" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G319" s="2" t="inlineStr">
+        <is>
+          <t>36b77e0a89c00685</t>
+        </is>
+      </c>
+      <c r="H319" s="2" t="inlineStr">
+        <is>
+          <t>401816428</t>
+        </is>
+      </c>
+      <c r="I319" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J319" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K319" s="2" t="inlineStr"/>
+      <c r="L319" s="2" t="inlineStr">
+        <is>
+          <t>0.581752</t>
+        </is>
+      </c>
+      <c r="M319" s="2" t="inlineStr"/>
+      <c r="N319" s="2" t="inlineStr"/>
+      <c r="O319" s="2" t="inlineStr">
+        <is>
+          <t>0.5594713656387665</t>
+        </is>
+      </c>
+      <c r="P319" s="2" t="inlineStr">
+        <is>
+          <t>0.557214</t>
+        </is>
+      </c>
+      <c r="Q319" s="2" t="inlineStr">
+        <is>
+          <t>0.02228063436123351</t>
+        </is>
+      </c>
+      <c r="R319" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:53.881975Z</t>
+        </is>
+      </c>
+      <c r="S319" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:40:00-0400</t>
+        </is>
+      </c>
+      <c r="T319" s="2" t="inlineStr"/>
+      <c r="U319" s="2" t="inlineStr"/>
+      <c r="V319" s="2" t="inlineStr"/>
+      <c r="W319" s="2" t="inlineStr"/>
+      <c r="X319" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y319" s="2" t="inlineStr"/>
+      <c r="Z319" s="2" t="inlineStr"/>
+      <c r="AA319" s="2" t="inlineStr"/>
+      <c r="AB319" s="2" t="inlineStr"/>
+      <c r="AC319" s="2" t="inlineStr"/>
+      <c r="AD319" s="2" t="inlineStr"/>
+      <c r="AE319" s="2" t="inlineStr"/>
+      <c r="AF319" s="2" t="inlineStr"/>
+      <c r="AG319" s="2" t="inlineStr"/>
+      <c r="AH319" s="2" t="inlineStr"/>
+      <c r="AI319" s="2" t="inlineStr"/>
+      <c r="AJ319" s="2" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>a8bcd75548df43b0</t>
+        </is>
+      </c>
+      <c r="B320" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E320" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F320" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G320" s="2" t="inlineStr">
+        <is>
+          <t>8e2973a0813de9d2</t>
+        </is>
+      </c>
+      <c r="H320" s="2" t="inlineStr">
+        <is>
+          <t>401816429</t>
+        </is>
+      </c>
+      <c r="I320" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J320" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K320" s="2" t="inlineStr"/>
+      <c r="L320" s="2" t="inlineStr">
+        <is>
+          <t>0.562475</t>
+        </is>
+      </c>
+      <c r="M320" s="2" t="inlineStr"/>
+      <c r="N320" s="2" t="inlineStr"/>
+      <c r="O320" s="2" t="inlineStr">
+        <is>
+          <t>0.6655518394648829</t>
+        </is>
+      </c>
+      <c r="P320" s="2" t="inlineStr">
+        <is>
+          <t>0.661692</t>
+        </is>
+      </c>
+      <c r="Q320" s="2" t="inlineStr">
+        <is>
+          <t>-0.103076839464883</t>
+        </is>
+      </c>
+      <c r="R320" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:53.313564Z</t>
+        </is>
+      </c>
+      <c r="S320" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:40:00-0400</t>
+        </is>
+      </c>
+      <c r="T320" s="2" t="inlineStr"/>
+      <c r="U320" s="2" t="inlineStr"/>
+      <c r="V320" s="2" t="inlineStr"/>
+      <c r="W320" s="2" t="inlineStr"/>
+      <c r="X320" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y320" s="2" t="inlineStr"/>
+      <c r="Z320" s="2" t="inlineStr"/>
+      <c r="AA320" s="2" t="inlineStr"/>
+      <c r="AB320" s="2" t="inlineStr"/>
+      <c r="AC320" s="2" t="inlineStr"/>
+      <c r="AD320" s="2" t="inlineStr"/>
+      <c r="AE320" s="2" t="inlineStr"/>
+      <c r="AF320" s="2" t="inlineStr"/>
+      <c r="AG320" s="2" t="inlineStr"/>
+      <c r="AH320" s="2" t="inlineStr"/>
+      <c r="AI320" s="2" t="inlineStr"/>
+      <c r="AJ320" s="2" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>0369358d03204a0b</t>
+        </is>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E321" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F321" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G321" s="2" t="inlineStr">
+        <is>
+          <t>b382714397f85937</t>
+        </is>
+      </c>
+      <c r="H321" s="2" t="inlineStr">
+        <is>
+          <t>401816426</t>
+        </is>
+      </c>
+      <c r="I321" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J321" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K321" s="2" t="inlineStr"/>
+      <c r="L321" s="2" t="inlineStr">
+        <is>
+          <t>0.531118</t>
+        </is>
+      </c>
+      <c r="M321" s="2" t="inlineStr"/>
+      <c r="N321" s="2" t="inlineStr"/>
+      <c r="O321" s="2" t="inlineStr">
+        <is>
+          <t>0.5555555555555556</t>
+        </is>
+      </c>
+      <c r="P321" s="2" t="inlineStr">
+        <is>
+          <t>0.552239</t>
+        </is>
+      </c>
+      <c r="Q321" s="2" t="inlineStr">
+        <is>
+          <t>-0.0244375555555556</t>
+        </is>
+      </c>
+      <c r="R321" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:54.963458Z</t>
+        </is>
+      </c>
+      <c r="S321" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T19:05:00-0400</t>
+        </is>
+      </c>
+      <c r="T321" s="2" t="inlineStr"/>
+      <c r="U321" s="2" t="inlineStr"/>
+      <c r="V321" s="2" t="inlineStr"/>
+      <c r="W321" s="2" t="inlineStr"/>
+      <c r="X321" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y321" s="2" t="inlineStr"/>
+      <c r="Z321" s="2" t="inlineStr"/>
+      <c r="AA321" s="2" t="inlineStr"/>
+      <c r="AB321" s="2" t="inlineStr"/>
+      <c r="AC321" s="2" t="inlineStr"/>
+      <c r="AD321" s="2" t="inlineStr"/>
+      <c r="AE321" s="2" t="inlineStr"/>
+      <c r="AF321" s="2" t="inlineStr"/>
+      <c r="AG321" s="2" t="inlineStr"/>
+      <c r="AH321" s="2" t="inlineStr"/>
+      <c r="AI321" s="2" t="inlineStr"/>
+      <c r="AJ321" s="2" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>0d57dfbb286a409d</t>
+        </is>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E322" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F322" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G322" s="2" t="inlineStr">
+        <is>
+          <t>8bd990e177da70c3</t>
+        </is>
+      </c>
+      <c r="H322" s="2" t="inlineStr">
+        <is>
+          <t>401816424</t>
+        </is>
+      </c>
+      <c r="I322" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J322" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K322" s="2" t="inlineStr"/>
+      <c r="L322" s="2" t="inlineStr">
+        <is>
+          <t>0.641185</t>
+        </is>
+      </c>
+      <c r="M322" s="2" t="inlineStr"/>
+      <c r="N322" s="2" t="inlineStr"/>
+      <c r="O322" s="2" t="inlineStr">
+        <is>
+          <t>0.5850622406639003</t>
+        </is>
+      </c>
+      <c r="P322" s="2" t="inlineStr">
+        <is>
+          <t>0.58209</t>
+        </is>
+      </c>
+      <c r="Q322" s="2" t="inlineStr">
+        <is>
+          <t>0.05612275933609967</t>
+        </is>
+      </c>
+      <c r="R322" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:55.953169Z</t>
+        </is>
+      </c>
+      <c r="S322" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T19:10:00-0400</t>
+        </is>
+      </c>
+      <c r="T322" s="2" t="inlineStr"/>
+      <c r="U322" s="2" t="inlineStr"/>
+      <c r="V322" s="2" t="inlineStr"/>
+      <c r="W322" s="2" t="inlineStr"/>
+      <c r="X322" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y322" s="2" t="inlineStr"/>
+      <c r="Z322" s="2" t="inlineStr"/>
+      <c r="AA322" s="2" t="inlineStr"/>
+      <c r="AB322" s="2" t="inlineStr"/>
+      <c r="AC322" s="2" t="inlineStr"/>
+      <c r="AD322" s="2" t="inlineStr"/>
+      <c r="AE322" s="2" t="inlineStr"/>
+      <c r="AF322" s="2" t="inlineStr"/>
+      <c r="AG322" s="2" t="inlineStr"/>
+      <c r="AH322" s="2" t="inlineStr"/>
+      <c r="AI322" s="2" t="inlineStr"/>
+      <c r="AJ322" s="2" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>8df16023b5cd4f26</t>
+        </is>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E323" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F323" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G323" s="2" t="inlineStr">
+        <is>
+          <t>e1b75023630563d1</t>
+        </is>
+      </c>
+      <c r="H323" s="2" t="inlineStr">
+        <is>
+          <t>401816425</t>
+        </is>
+      </c>
+      <c r="I323" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J323" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K323" s="2" t="inlineStr"/>
+      <c r="L323" s="2" t="inlineStr">
+        <is>
+          <t>0.633651</t>
+        </is>
+      </c>
+      <c r="M323" s="2" t="inlineStr"/>
+      <c r="N323" s="2" t="inlineStr"/>
+      <c r="O323" s="2" t="inlineStr">
+        <is>
+          <t>0.715099715099715</t>
+        </is>
+      </c>
+      <c r="P323" s="2" t="inlineStr">
+        <is>
+          <t>0.711443</t>
+        </is>
+      </c>
+      <c r="Q323" s="2" t="inlineStr">
+        <is>
+          <t>-0.08144871509971507</t>
+        </is>
+      </c>
+      <c r="R323" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:55.473435Z</t>
+        </is>
+      </c>
+      <c r="S323" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T19:10:00-0400</t>
+        </is>
+      </c>
+      <c r="T323" s="2" t="inlineStr"/>
+      <c r="U323" s="2" t="inlineStr"/>
+      <c r="V323" s="2" t="inlineStr"/>
+      <c r="W323" s="2" t="inlineStr"/>
+      <c r="X323" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y323" s="2" t="inlineStr"/>
+      <c r="Z323" s="2" t="inlineStr"/>
+      <c r="AA323" s="2" t="inlineStr"/>
+      <c r="AB323" s="2" t="inlineStr"/>
+      <c r="AC323" s="2" t="inlineStr"/>
+      <c r="AD323" s="2" t="inlineStr"/>
+      <c r="AE323" s="2" t="inlineStr"/>
+      <c r="AF323" s="2" t="inlineStr"/>
+      <c r="AG323" s="2" t="inlineStr"/>
+      <c r="AH323" s="2" t="inlineStr"/>
+      <c r="AI323" s="2" t="inlineStr"/>
+      <c r="AJ323" s="2" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>55626f9b1cc84979</t>
+        </is>
+      </c>
+      <c r="B324" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C324" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E324" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F324" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G324" s="2" t="inlineStr">
+        <is>
+          <t>53df13bab12c4582</t>
+        </is>
+      </c>
+      <c r="H324" s="2" t="inlineStr">
+        <is>
+          <t>401816432</t>
+        </is>
+      </c>
+      <c r="I324" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J324" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K324" s="2" t="inlineStr"/>
+      <c r="L324" s="2" t="inlineStr">
+        <is>
+          <t>0.522033</t>
+        </is>
+      </c>
+      <c r="M324" s="2" t="inlineStr"/>
+      <c r="N324" s="2" t="inlineStr"/>
+      <c r="O324" s="2" t="inlineStr">
+        <is>
+          <t>0.4291845493562232</t>
+        </is>
+      </c>
+      <c r="P324" s="2" t="inlineStr">
+        <is>
+          <t>0.427861</t>
+        </is>
+      </c>
+      <c r="Q324" s="2" t="inlineStr">
+        <is>
+          <t>0.09284845064377678</t>
+        </is>
+      </c>
+      <c r="R324" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:57.437825Z</t>
+        </is>
+      </c>
+      <c r="S324" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T19:40:00-0400</t>
+        </is>
+      </c>
+      <c r="T324" s="2" t="inlineStr"/>
+      <c r="U324" s="2" t="inlineStr"/>
+      <c r="V324" s="2" t="inlineStr"/>
+      <c r="W324" s="2" t="inlineStr"/>
+      <c r="X324" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y324" s="2" t="inlineStr"/>
+      <c r="Z324" s="2" t="inlineStr"/>
+      <c r="AA324" s="2" t="inlineStr"/>
+      <c r="AB324" s="2" t="inlineStr"/>
+      <c r="AC324" s="2" t="inlineStr"/>
+      <c r="AD324" s="2" t="inlineStr"/>
+      <c r="AE324" s="2" t="inlineStr"/>
+      <c r="AF324" s="2" t="inlineStr"/>
+      <c r="AG324" s="2" t="inlineStr"/>
+      <c r="AH324" s="2" t="inlineStr"/>
+      <c r="AI324" s="2" t="inlineStr"/>
+      <c r="AJ324" s="2" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
+          <t>b216031ab5ef493b</t>
+        </is>
+      </c>
+      <c r="B325" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C325" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D325" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E325" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F325" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G325" s="2" t="inlineStr">
+        <is>
+          <t>6930bf181d0a558c</t>
+        </is>
+      </c>
+      <c r="H325" s="2" t="inlineStr">
+        <is>
+          <t>401816434</t>
+        </is>
+      </c>
+      <c r="I325" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J325" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K325" s="2" t="inlineStr"/>
+      <c r="L325" s="2" t="inlineStr">
+        <is>
+          <t>0.651659</t>
+        </is>
+      </c>
+      <c r="M325" s="2" t="inlineStr"/>
+      <c r="N325" s="2" t="inlineStr"/>
+      <c r="O325" s="2" t="inlineStr">
+        <is>
+          <t>0.6197718631178707</t>
+        </is>
+      </c>
+      <c r="P325" s="2" t="inlineStr">
+        <is>
+          <t>0.616915</t>
+        </is>
+      </c>
+      <c r="Q325" s="2" t="inlineStr">
+        <is>
+          <t>0.0318871368821293</t>
+        </is>
+      </c>
+      <c r="R325" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:56.444164Z</t>
+        </is>
+      </c>
+      <c r="S325" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T19:40:00-0400</t>
+        </is>
+      </c>
+      <c r="T325" s="2" t="inlineStr"/>
+      <c r="U325" s="2" t="inlineStr"/>
+      <c r="V325" s="2" t="inlineStr"/>
+      <c r="W325" s="2" t="inlineStr"/>
+      <c r="X325" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y325" s="2" t="inlineStr"/>
+      <c r="Z325" s="2" t="inlineStr"/>
+      <c r="AA325" s="2" t="inlineStr"/>
+      <c r="AB325" s="2" t="inlineStr"/>
+      <c r="AC325" s="2" t="inlineStr"/>
+      <c r="AD325" s="2" t="inlineStr"/>
+      <c r="AE325" s="2" t="inlineStr"/>
+      <c r="AF325" s="2" t="inlineStr"/>
+      <c r="AG325" s="2" t="inlineStr"/>
+      <c r="AH325" s="2" t="inlineStr"/>
+      <c r="AI325" s="2" t="inlineStr"/>
+      <c r="AJ325" s="2" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>0a05673eba8c47ba</t>
+        </is>
+      </c>
+      <c r="B326" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E326" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F326" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G326" s="2" t="inlineStr">
+        <is>
+          <t>db25d2479efd20e9</t>
+        </is>
+      </c>
+      <c r="H326" s="2" t="inlineStr">
+        <is>
+          <t>401816431</t>
+        </is>
+      </c>
+      <c r="I326" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J326" s="2" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="K326" s="2" t="inlineStr"/>
+      <c r="L326" s="2" t="inlineStr">
+        <is>
+          <t>0.532629</t>
+        </is>
+      </c>
+      <c r="M326" s="2" t="inlineStr"/>
+      <c r="N326" s="2" t="inlineStr"/>
+      <c r="O326" s="2" t="inlineStr">
+        <is>
+          <t>0.6153846153846154</t>
+        </is>
+      </c>
+      <c r="P326" s="2" t="inlineStr">
+        <is>
+          <t>0.61194</t>
+        </is>
+      </c>
+      <c r="Q326" s="2" t="inlineStr">
+        <is>
+          <t>-0.0827556153846154</t>
+        </is>
+      </c>
+      <c r="R326" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:57.775453Z</t>
+        </is>
+      </c>
+      <c r="S326" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T20:10:00-0400</t>
+        </is>
+      </c>
+      <c r="T326" s="2" t="inlineStr"/>
+      <c r="U326" s="2" t="inlineStr"/>
+      <c r="V326" s="2" t="inlineStr"/>
+      <c r="W326" s="2" t="inlineStr"/>
+      <c r="X326" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y326" s="2" t="inlineStr"/>
+      <c r="Z326" s="2" t="inlineStr"/>
+      <c r="AA326" s="2" t="inlineStr"/>
+      <c r="AB326" s="2" t="inlineStr"/>
+      <c r="AC326" s="2" t="inlineStr"/>
+      <c r="AD326" s="2" t="inlineStr"/>
+      <c r="AE326" s="2" t="inlineStr"/>
+      <c r="AF326" s="2" t="inlineStr"/>
+      <c r="AG326" s="2" t="inlineStr"/>
+      <c r="AH326" s="2" t="inlineStr"/>
+      <c r="AI326" s="2" t="inlineStr"/>
+      <c r="AJ326" s="2" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="inlineStr">
+        <is>
+          <t>128b0e95c10545ac</t>
+        </is>
+      </c>
+      <c r="B327" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E327" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F327" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G327" s="2" t="inlineStr">
+        <is>
+          <t>014888ea3e3e3318</t>
+        </is>
+      </c>
+      <c r="H327" s="2" t="inlineStr">
+        <is>
+          <t>401816430</t>
+        </is>
+      </c>
+      <c r="I327" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J327" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K327" s="2" t="inlineStr"/>
+      <c r="L327" s="2" t="inlineStr">
+        <is>
+          <t>0.551691</t>
+        </is>
+      </c>
+      <c r="M327" s="2" t="inlineStr"/>
+      <c r="N327" s="2" t="inlineStr"/>
+      <c r="O327" s="2" t="inlineStr">
+        <is>
+          <t>0.5798319327731092</t>
+        </is>
+      </c>
+      <c r="P327" s="2" t="inlineStr">
+        <is>
+          <t>0.577114</t>
+        </is>
+      </c>
+      <c r="Q327" s="2" t="inlineStr">
+        <is>
+          <t>-0.02814093277310914</t>
+        </is>
+      </c>
+      <c r="R327" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:58.624050Z</t>
+        </is>
+      </c>
+      <c r="S327" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T20:15:00-0400</t>
+        </is>
+      </c>
+      <c r="T327" s="2" t="inlineStr"/>
+      <c r="U327" s="2" t="inlineStr"/>
+      <c r="V327" s="2" t="inlineStr"/>
+      <c r="W327" s="2" t="inlineStr"/>
+      <c r="X327" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y327" s="2" t="inlineStr"/>
+      <c r="Z327" s="2" t="inlineStr"/>
+      <c r="AA327" s="2" t="inlineStr"/>
+      <c r="AB327" s="2" t="inlineStr"/>
+      <c r="AC327" s="2" t="inlineStr"/>
+      <c r="AD327" s="2" t="inlineStr"/>
+      <c r="AE327" s="2" t="inlineStr"/>
+      <c r="AF327" s="2" t="inlineStr"/>
+      <c r="AG327" s="2" t="inlineStr"/>
+      <c r="AH327" s="2" t="inlineStr"/>
+      <c r="AI327" s="2" t="inlineStr"/>
+      <c r="AJ327" s="2" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>955a1482baa548b2</t>
+        </is>
+      </c>
+      <c r="B328" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E328" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F328" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G328" s="2" t="inlineStr">
+        <is>
+          <t>cf5d809f58d18264</t>
+        </is>
+      </c>
+      <c r="H328" s="2" t="inlineStr">
+        <is>
+          <t>401816433</t>
+        </is>
+      </c>
+      <c r="I328" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J328" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K328" s="2" t="inlineStr"/>
+      <c r="L328" s="2" t="inlineStr">
+        <is>
+          <t>0.667145</t>
+        </is>
+      </c>
+      <c r="M328" s="2" t="inlineStr"/>
+      <c r="N328" s="2" t="inlineStr"/>
+      <c r="O328" s="2" t="inlineStr">
+        <is>
+          <t>0.6153846153846154</t>
+        </is>
+      </c>
+      <c r="P328" s="2" t="inlineStr">
+        <is>
+          <t>0.61194</t>
+        </is>
+      </c>
+      <c r="Q328" s="2" t="inlineStr">
+        <is>
+          <t>0.05176038461538457</t>
+        </is>
+      </c>
+      <c r="R328" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:59.237881Z</t>
+        </is>
+      </c>
+      <c r="S328" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T20:15:00-0400</t>
+        </is>
+      </c>
+      <c r="T328" s="2" t="inlineStr"/>
+      <c r="U328" s="2" t="inlineStr"/>
+      <c r="V328" s="2" t="inlineStr"/>
+      <c r="W328" s="2" t="inlineStr"/>
+      <c r="X328" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y328" s="2" t="inlineStr"/>
+      <c r="Z328" s="2" t="inlineStr"/>
+      <c r="AA328" s="2" t="inlineStr"/>
+      <c r="AB328" s="2" t="inlineStr"/>
+      <c r="AC328" s="2" t="inlineStr"/>
+      <c r="AD328" s="2" t="inlineStr"/>
+      <c r="AE328" s="2" t="inlineStr"/>
+      <c r="AF328" s="2" t="inlineStr"/>
+      <c r="AG328" s="2" t="inlineStr"/>
+      <c r="AH328" s="2" t="inlineStr"/>
+      <c r="AI328" s="2" t="inlineStr"/>
+      <c r="AJ328" s="2" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>75f5ed3c3c2647f1</t>
+        </is>
+      </c>
+      <c r="B329" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E329" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F329" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G329" s="2" t="inlineStr">
+        <is>
+          <t>f41cdedf84b1bab8</t>
+        </is>
+      </c>
+      <c r="H329" s="2" t="inlineStr">
+        <is>
+          <t>401816436</t>
+        </is>
+      </c>
+      <c r="I329" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J329" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K329" s="2" t="inlineStr"/>
+      <c r="L329" s="2" t="inlineStr">
+        <is>
+          <t>0.586422</t>
+        </is>
+      </c>
+      <c r="M329" s="2" t="inlineStr"/>
+      <c r="N329" s="2" t="inlineStr"/>
+      <c r="O329" s="2" t="inlineStr">
+        <is>
+          <t>0.5260663507109005</t>
+        </is>
+      </c>
+      <c r="P329" s="2" t="inlineStr">
+        <is>
+          <t>0.522388</t>
+        </is>
+      </c>
+      <c r="Q329" s="2" t="inlineStr">
+        <is>
+          <t>0.06035564928909953</t>
+        </is>
+      </c>
+      <c r="R329" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:27:59.634473Z</t>
+        </is>
+      </c>
+      <c r="S329" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T21:40:00-0400</t>
+        </is>
+      </c>
+      <c r="T329" s="2" t="inlineStr"/>
+      <c r="U329" s="2" t="inlineStr"/>
+      <c r="V329" s="2" t="inlineStr"/>
+      <c r="W329" s="2" t="inlineStr"/>
+      <c r="X329" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y329" s="2" t="inlineStr"/>
+      <c r="Z329" s="2" t="inlineStr"/>
+      <c r="AA329" s="2" t="inlineStr"/>
+      <c r="AB329" s="2" t="inlineStr"/>
+      <c r="AC329" s="2" t="inlineStr"/>
+      <c r="AD329" s="2" t="inlineStr"/>
+      <c r="AE329" s="2" t="inlineStr"/>
+      <c r="AF329" s="2" t="inlineStr"/>
+      <c r="AG329" s="2" t="inlineStr"/>
+      <c r="AH329" s="2" t="inlineStr"/>
+      <c r="AI329" s="2" t="inlineStr"/>
+      <c r="AJ329" s="2" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>f493f2e498264692</t>
+        </is>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E330" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F330" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G330" s="2" t="inlineStr">
+        <is>
+          <t>807bfd9a83666e43</t>
+        </is>
+      </c>
+      <c r="H330" s="2" t="inlineStr">
+        <is>
+          <t>401816437</t>
+        </is>
+      </c>
+      <c r="I330" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J330" s="2" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="K330" s="2" t="inlineStr"/>
+      <c r="L330" s="2" t="inlineStr">
+        <is>
+          <t>0.527996</t>
+        </is>
+      </c>
+      <c r="M330" s="2" t="inlineStr"/>
+      <c r="N330" s="2" t="inlineStr"/>
+      <c r="O330" s="2" t="inlineStr">
+        <is>
+          <t>0.6197718631178707</t>
+        </is>
+      </c>
+      <c r="P330" s="2" t="inlineStr">
+        <is>
+          <t>0.616915</t>
+        </is>
+      </c>
+      <c r="Q330" s="2" t="inlineStr">
+        <is>
+          <t>-0.09177586311787067</t>
+        </is>
+      </c>
+      <c r="R330" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:28:00.536930Z</t>
+        </is>
+      </c>
+      <c r="S330" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T21:40:00-0400</t>
+        </is>
+      </c>
+      <c r="T330" s="2" t="inlineStr"/>
+      <c r="U330" s="2" t="inlineStr"/>
+      <c r="V330" s="2" t="inlineStr"/>
+      <c r="W330" s="2" t="inlineStr"/>
+      <c r="X330" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y330" s="2" t="inlineStr"/>
+      <c r="Z330" s="2" t="inlineStr"/>
+      <c r="AA330" s="2" t="inlineStr"/>
+      <c r="AB330" s="2" t="inlineStr"/>
+      <c r="AC330" s="2" t="inlineStr"/>
+      <c r="AD330" s="2" t="inlineStr"/>
+      <c r="AE330" s="2" t="inlineStr"/>
+      <c r="AF330" s="2" t="inlineStr"/>
+      <c r="AG330" s="2" t="inlineStr"/>
+      <c r="AH330" s="2" t="inlineStr"/>
+      <c r="AI330" s="2" t="inlineStr"/>
+      <c r="AJ330" s="2" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>9978fb6eb7ea49aa</t>
+        </is>
+      </c>
+      <c r="B331" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
+        <is>
+          <t>mlb-moneyline-elo-trend-lr</t>
+        </is>
+      </c>
+      <c r="D331" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="E331" s="2" t="inlineStr">
+        <is>
+          <t>6a5c79541b0e50cb9f7318270e63d5ccc65cbd7bc53a019748ff772d49de5075</t>
+        </is>
+      </c>
+      <c r="F331" s="2" t="inlineStr">
+        <is>
+          <t>mlb-elo-trend-lr-v8</t>
+        </is>
+      </c>
+      <c r="G331" s="2" t="inlineStr">
+        <is>
+          <t>cf9d26fcd493bc83</t>
+        </is>
+      </c>
+      <c r="H331" s="2" t="inlineStr">
+        <is>
+          <t>401816438</t>
+        </is>
+      </c>
+      <c r="I331" s="2" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="J331" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="K331" s="2" t="inlineStr"/>
+      <c r="L331" s="2" t="inlineStr">
+        <is>
+          <t>0.556751</t>
+        </is>
+      </c>
+      <c r="M331" s="2" t="inlineStr"/>
+      <c r="N331" s="2" t="inlineStr"/>
+      <c r="O331" s="2" t="inlineStr">
+        <is>
+          <t>0.5192307692307692</t>
+        </is>
+      </c>
+      <c r="P331" s="2" t="inlineStr">
+        <is>
+          <t>0.517413</t>
+        </is>
+      </c>
+      <c r="Q331" s="2" t="inlineStr">
+        <is>
+          <t>0.03752023076923083</t>
+        </is>
+      </c>
+      <c r="R331" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:28:01.370150Z</t>
+        </is>
+      </c>
+      <c r="S331" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07T21:45:00-0400</t>
+        </is>
+      </c>
+      <c r="T331" s="2" t="inlineStr"/>
+      <c r="U331" s="2" t="inlineStr"/>
+      <c r="V331" s="2" t="inlineStr"/>
+      <c r="W331" s="2" t="inlineStr"/>
+      <c r="X331" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y331" s="2" t="inlineStr"/>
+      <c r="Z331" s="2" t="inlineStr"/>
+      <c r="AA331" s="2" t="inlineStr"/>
+      <c r="AB331" s="2" t="inlineStr"/>
+      <c r="AC331" s="2" t="inlineStr"/>
+      <c r="AD331" s="2" t="inlineStr"/>
+      <c r="AE331" s="2" t="inlineStr"/>
+      <c r="AF331" s="2" t="inlineStr"/>
+      <c r="AG331" s="2" t="inlineStr"/>
+      <c r="AH331" s="2" t="inlineStr"/>
+      <c r="AI331" s="2" t="inlineStr"/>
+      <c r="AJ331" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ318"/>
+  <autoFilter ref="A1:AJ331"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>